<commit_message>
cambio pequeño de etl y kdd listo
</commit_message>
<xml_diff>
--- a/etl/datos_limpios.xlsx
+++ b/etl/datos_limpios.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>difficulty_level</t>
+          <t>duration_level</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>para la masa:, 3 tazas de harina, 70 grs de manteca derretida, 1 taza de leche tibia, 1 cucharadita de polvos de hornear, 1 cucharadita de sal, para el pino, 2 a 3 cucharadas de aceite maravilla o canola, 2 cebollas picadas en cuadros, 1/2 kilo de surtido de mariscos, 1 cucharadita de ají color (puede reemplazar por paprika), 1 cucharadita de ají en pasta, 1/2 cucharadita de orégano, sal a gusto</t>
+          <t>Para la masa:, 3 tazas de harina, 70 grs de manteca derretida, 1 taza de leche tibia, 1 cucharadita de polvos de hornear, 1 cucharadita de sal, para el pino, 2 a 3 cucharadas de aceite maravilla o canola, 2 cebollas picadas en cuadros, 1/2 kilo de surtido de mariscos, 1 cucharadita de ají color (puede reemplazar por paprika), 1 cucharadita de ají en pasta, 1/2 cucharadita de orégano, sal a gusto</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Nan</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Nan</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">

</xml_diff>